<commit_message>
Updated MYS_grids_kan model - 2026-05-06 23:14
</commit_message>
<xml_diff>
--- a/VerveStacks_MYS_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_MYS_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_MYS_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A84B72E7-AE78-4DD1-965F-6BED7CC3E06E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{97B4886F-8B0C-4C28-8D8C-1111EC770174}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3847,7 +3847,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BBCA4F9-EBB7-41D9-A241-66975B3FC148}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50CC8F0C-1037-46E3-A85E-B2CF841F6ED4}">
   <dimension ref="B9:H215"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -24098,7 +24098,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0D57DEE-4F66-46FA-8C39-98E937A0A6A2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99E0A671-08FB-443A-86CF-4137A0B2CDFB}">
   <dimension ref="B9:L215"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>